<commit_message>
TENCON 2026 paper deleted from news and publications
</commit_message>
<xml_diff>
--- a/data/news.xlsx
+++ b/data/news.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10821"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jitendra/Git Projects/jitendrakv.github.io/data/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Git Projects\jitendrakv.github.io\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F19D6CAD-941B-CD49-B436-7C2B668A1B8B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6F8C6979-B4DD-40A5-AD98-1A38D5875DAA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="140" yWindow="760" windowWidth="20500" windowHeight="18880" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Instructions" sheetId="1" r:id="rId1"/>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="109" uniqueCount="83">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="106" uniqueCount="81">
   <si>
     <t>Year</t>
   </si>
@@ -54,13 +54,6 @@
   </si>
   <si>
     <t>Publication</t>
-  </si>
-  <si>
-    <t>Collaborative Learning Enabled Workload
-Prediction Model for Large-Scale Cloud Environments</t>
-  </si>
-  <si>
-    <t>is accepted for presentation in IEEE TENCON-2026</t>
   </si>
   <si>
     <t>Special session on "Advances in Artificial Intelligence: Models, Systems, and Applications"</t>
@@ -696,32 +689,32 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:A5"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="105" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:1" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A2" s="2"/>
+    </row>
+    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A3" s="2" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A4" s="2" t="s">
         <v>72</v>
       </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A2" s="2"/>
-    </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A3" s="2" t="s">
+    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A5" s="2" t="s">
         <v>73</v>
-      </c>
-    </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A4" s="2" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A5" s="2" t="s">
-        <v>75</v>
       </c>
     </row>
   </sheetData>
@@ -731,8 +724,8 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:E32"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <dimension ref="A1:E31"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="8" customWidth="1"/>
     <col min="2" max="2" width="18" customWidth="1"/>
@@ -740,7 +733,7 @@
     <col min="5" max="5" width="34" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -757,7 +750,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:5" ht="32" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:5" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="4">
         <v>2026</v>
       </c>
@@ -774,7 +767,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="3" spans="1:5" ht="40" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:5" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="4">
         <v>2026</v>
       </c>
@@ -782,46 +775,46 @@
         <v>9</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="E3" s="4"/>
     </row>
-    <row r="4" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="4">
         <v>2026</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="C4" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="D4" s="4" t="s">
+      <c r="D4" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="E4" s="4"/>
-    </row>
-    <row r="5" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="E4" s="5" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="4">
         <v>2026</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="D5" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="E5" s="5" t="s">
+      <c r="D5" s="4" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="6" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="E5" s="4"/>
+    </row>
+    <row r="6" spans="1:5" ht="45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="4">
         <v>2026</v>
       </c>
@@ -836,7 +829,7 @@
       </c>
       <c r="E6" s="4"/>
     </row>
-    <row r="7" spans="1:5" ht="45" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:5" ht="45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="4">
         <v>2026</v>
       </c>
@@ -851,87 +844,87 @@
       </c>
       <c r="E7" s="4"/>
     </row>
-    <row r="8" spans="1:5" ht="45" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:5" ht="45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="4">
         <v>2026</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="C8" s="4" t="s">
-        <v>20</v>
+        <v>55</v>
+      </c>
+      <c r="C8" s="7" t="s">
+        <v>74</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>21</v>
+        <v>80</v>
       </c>
       <c r="E8" s="4"/>
     </row>
-    <row r="9" spans="1:5" ht="45" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="4">
         <v>2026</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>57</v>
-      </c>
-      <c r="C9" s="7" t="s">
-        <v>76</v>
+        <v>10</v>
+      </c>
+      <c r="C9" s="4" t="s">
+        <v>20</v>
       </c>
       <c r="D9" s="4" t="s">
-        <v>82</v>
+        <v>21</v>
       </c>
       <c r="E9" s="4"/>
     </row>
-    <row r="10" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="4">
         <v>2026</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>10</v>
+        <v>55</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>22</v>
+        <v>75</v>
       </c>
       <c r="D10" s="4" t="s">
-        <v>23</v>
+        <v>80</v>
       </c>
       <c r="E10" s="4"/>
     </row>
-    <row r="11" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="4">
         <v>2026</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>57</v>
+        <v>10</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>77</v>
+        <v>22</v>
       </c>
       <c r="D11" s="4" t="s">
-        <v>82</v>
+        <v>23</v>
       </c>
       <c r="E11" s="4"/>
     </row>
-    <row r="12" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="4">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>10</v>
+        <v>24</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="D12" s="4" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="E12" s="4"/>
     </row>
-    <row r="13" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:5" ht="45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="4">
         <v>2025</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>26</v>
+        <v>10</v>
       </c>
       <c r="C13" s="4" t="s">
         <v>27</v>
@@ -941,7 +934,7 @@
       </c>
       <c r="E13" s="4"/>
     </row>
-    <row r="14" spans="1:5" ht="45" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="4">
         <v>2025</v>
       </c>
@@ -956,7 +949,7 @@
       </c>
       <c r="E14" s="4"/>
     </row>
-    <row r="15" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:5" ht="45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="4">
         <v>2025</v>
       </c>
@@ -971,7 +964,7 @@
       </c>
       <c r="E15" s="4"/>
     </row>
-    <row r="16" spans="1:5" ht="45" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="4">
         <v>2025</v>
       </c>
@@ -986,7 +979,7 @@
       </c>
       <c r="E16" s="4"/>
     </row>
-    <row r="17" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="4">
         <v>2025</v>
       </c>
@@ -1001,37 +994,39 @@
       </c>
       <c r="E17" s="4"/>
     </row>
-    <row r="18" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="4">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="B18" s="4" t="s">
-        <v>10</v>
+        <v>24</v>
       </c>
       <c r="C18" s="4" t="s">
-        <v>37</v>
+        <v>76</v>
       </c>
       <c r="D18" s="4" t="s">
-        <v>38</v>
+        <v>77</v>
       </c>
       <c r="E18" s="4"/>
     </row>
-    <row r="19" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:5" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="4">
         <v>2024</v>
       </c>
       <c r="B19" s="4" t="s">
-        <v>26</v>
+        <v>10</v>
       </c>
       <c r="C19" s="4" t="s">
-        <v>78</v>
+        <v>37</v>
       </c>
       <c r="D19" s="4" t="s">
-        <v>79</v>
-      </c>
-      <c r="E19" s="4"/>
-    </row>
-    <row r="20" spans="1:5" ht="60" customHeight="1" x14ac:dyDescent="0.2">
+        <v>38</v>
+      </c>
+      <c r="E19" s="4" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="4">
         <v>2024</v>
       </c>
@@ -1039,21 +1034,19 @@
         <v>10</v>
       </c>
       <c r="C20" s="4" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="D20" s="4" t="s">
-        <v>40</v>
-      </c>
-      <c r="E20" s="4" t="s">
         <v>41</v>
       </c>
-    </row>
-    <row r="21" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="E20" s="4"/>
+    </row>
+    <row r="21" spans="1:5" ht="45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="4">
-        <v>2024</v>
+        <v>2023</v>
       </c>
       <c r="B21" s="4" t="s">
-        <v>10</v>
+        <v>24</v>
       </c>
       <c r="C21" s="4" t="s">
         <v>42</v>
@@ -1063,12 +1056,12 @@
       </c>
       <c r="E21" s="4"/>
     </row>
-    <row r="22" spans="1:5" ht="45" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:5" ht="45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="4">
         <v>2023</v>
       </c>
       <c r="B22" s="4" t="s">
-        <v>26</v>
+        <v>10</v>
       </c>
       <c r="C22" s="4" t="s">
         <v>44</v>
@@ -1078,7 +1071,7 @@
       </c>
       <c r="E22" s="4"/>
     </row>
-    <row r="23" spans="1:5" ht="45" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="4">
         <v>2023</v>
       </c>
@@ -1093,61 +1086,61 @@
       </c>
       <c r="E23" s="4"/>
     </row>
-    <row r="24" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:5" ht="90" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="4">
         <v>2023</v>
       </c>
       <c r="B24" s="4" t="s">
-        <v>10</v>
+        <v>48</v>
       </c>
       <c r="C24" s="4" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="D24" s="4" t="s">
-        <v>49</v>
-      </c>
-      <c r="E24" s="4"/>
-    </row>
-    <row r="25" spans="1:5" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+        <v>50</v>
+      </c>
+      <c r="E24" s="4" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" ht="45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="4">
         <v>2023</v>
       </c>
       <c r="B25" s="4" t="s">
-        <v>50</v>
+        <v>24</v>
       </c>
       <c r="C25" s="4" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="D25" s="4" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="E25" s="4" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="26" spans="1:5" ht="45" customHeight="1" x14ac:dyDescent="0.2">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" ht="27" x14ac:dyDescent="0.25">
       <c r="A26" s="4">
         <v>2023</v>
       </c>
       <c r="B26" s="4" t="s">
-        <v>26</v>
+        <v>55</v>
       </c>
       <c r="C26" s="4" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="D26" s="4" t="s">
-        <v>55</v>
-      </c>
-      <c r="E26" s="4" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.2">
+        <v>57</v>
+      </c>
+      <c r="E26" s="4"/>
+    </row>
+    <row r="27" spans="1:5" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="4">
         <v>2023</v>
       </c>
       <c r="B27" s="4" t="s">
-        <v>57</v>
+        <v>48</v>
       </c>
       <c r="C27" s="4" t="s">
         <v>58</v>
@@ -1155,31 +1148,31 @@
       <c r="D27" s="4" t="s">
         <v>59</v>
       </c>
-      <c r="E27" s="4"/>
-    </row>
-    <row r="28" spans="1:5" ht="60" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="E27" s="4" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A28" s="4">
         <v>2023</v>
       </c>
       <c r="B28" s="4" t="s">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="C28" s="4" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="D28" s="4" t="s">
-        <v>61</v>
-      </c>
-      <c r="E28" s="4" t="s">
         <v>62</v>
       </c>
-    </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="E28" s="4"/>
+    </row>
+    <row r="29" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="4">
         <v>2023</v>
       </c>
       <c r="B29" s="4" t="s">
-        <v>57</v>
+        <v>48</v>
       </c>
       <c r="C29" s="4" t="s">
         <v>63</v>
@@ -1187,31 +1180,31 @@
       <c r="D29" s="4" t="s">
         <v>64</v>
       </c>
-      <c r="E29" s="4"/>
-    </row>
-    <row r="30" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="E29" s="4" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="4">
         <v>2023</v>
       </c>
       <c r="B30" s="4" t="s">
-        <v>50</v>
+        <v>10</v>
       </c>
       <c r="C30" s="4" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="D30" s="4" t="s">
-        <v>66</v>
-      </c>
-      <c r="E30" s="4" t="s">
         <v>67</v>
       </c>
-    </row>
-    <row r="31" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="E30" s="4"/>
+    </row>
+    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A31" s="4">
         <v>2023</v>
       </c>
       <c r="B31" s="4" t="s">
-        <v>10</v>
+        <v>55</v>
       </c>
       <c r="C31" s="4" t="s">
         <v>68</v>
@@ -1221,24 +1214,9 @@
       </c>
       <c r="E31" s="4"/>
     </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A32" s="4">
-        <v>2023</v>
-      </c>
-      <c r="B32" s="4" t="s">
-        <v>57</v>
-      </c>
-      <c r="C32" s="4" t="s">
-        <v>70</v>
-      </c>
-      <c r="D32" s="4" t="s">
-        <v>71</v>
-      </c>
-      <c r="E32" s="4"/>
-    </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" sqref="B8:B508" xr:uid="{00000000-0002-0000-0100-000000000000}">
+    <dataValidation type="list" allowBlank="1" sqref="B7:B507" xr:uid="{00000000-0002-0000-0100-000000000000}">
       <formula1>"Research Paper,Journal Paper,Conference Paper,Conference,Invited Talk,Call for Papers,News Update"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>